<commit_message>
Add GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/src/main/resources/priceReport.xlsx
+++ b/src/main/resources/priceReport.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>Product Name</t>
   </si>
@@ -48,12 +48,6 @@
   </si>
   <si>
     <t>https://www.amazon.in/dp/B0FBKCDQ9X</t>
-  </si>
-  <si>
-    <t>Anarkali Kurti</t>
-  </si>
-  <si>
-    <t>https://www.amazon.in/dp/B0H1R6YTDV</t>
   </si>
   <si>
     <t>Door mat</t>
@@ -79,19 +73,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <u val="single"/>
-      <color indexed="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -150,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -158,14 +146,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.39453125" customWidth="true" bestFit="true"/>
@@ -248,10 +235,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>1699.0</v>
+        <v>199.0</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>6</v>
@@ -265,10 +252,10 @@
         <v>14</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>100.0</v>
+        <v>15000.0</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>199.0</v>
+        <v>16999.0</v>
       </c>
       <c r="D6" t="s" s="0">
         <v>6</v>
@@ -282,33 +269,16 @@
         <v>16</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>15000.0</v>
+        <v>4000.0</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>16999.0</v>
+        <v>5999.0</v>
       </c>
       <c r="D7" t="s" s="0">
         <v>6</v>
       </c>
       <c r="E7" t="s" s="6">
         <v>17</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="B8" t="n" s="0">
-        <v>4000.0</v>
-      </c>
-      <c r="C8" t="n" s="0">
-        <v>5999.0</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="E8" t="s" s="7">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -319,7 +289,6 @@
     <hyperlink ref="E5" r:id="rId4"/>
     <hyperlink ref="E6" r:id="rId5"/>
     <hyperlink ref="E7" r:id="rId6"/>
-    <hyperlink ref="E8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Add reporting framework, notifications, dashboard and Jenkins scheduling
</commit_message>
<xml_diff>
--- a/src/main/resources/priceReport.xlsx
+++ b/src/main/resources/priceReport.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>Product Name</t>
   </si>
@@ -38,12 +38,6 @@
     <t>https://www.amazon.in/dp/B0DZ2RMZQF</t>
   </si>
   <si>
-    <t>Casual wide leg pant</t>
-  </si>
-  <si>
-    <t>https://www.amazon.in/dp/B0GL8JRB3K</t>
-  </si>
-  <si>
     <t>Cut shoe</t>
   </si>
   <si>
@@ -63,6 +57,9 @@
   </si>
   <si>
     <t>Shoe rack</t>
+  </si>
+  <si>
+    <t>DROPPED</t>
   </si>
   <si>
     <t>https://www.amazon.in/dp/B0GXQ8Z3YB</t>
@@ -73,19 +70,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <u val="single"/>
-      <color indexed="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -138,27 +129,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="17.39453125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="12.7890625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="10.51953125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="11.49609375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="7.1640625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="8.73828125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="34.984375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -201,10 +191,10 @@
         <v>8</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>450.0</v>
+        <v>700.0</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>595.0</v>
+        <v>1098.0</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>6</v>
@@ -218,10 +208,10 @@
         <v>10</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>700.0</v>
+        <v>100.0</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>1099.0</v>
+        <v>249.0</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>6</v>
@@ -235,10 +225,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>100.0</v>
+        <v>15000.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>199.0</v>
+        <v>16999.0</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>6</v>
@@ -252,33 +242,16 @@
         <v>14</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>15000.0</v>
+        <v>4000.0</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>16999.0</v>
+        <v>2999.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E6" t="s" s="5">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
         <v>16</v>
-      </c>
-      <c r="B7" t="n" s="0">
-        <v>4000.0</v>
-      </c>
-      <c r="C7" t="n" s="0">
-        <v>5999.0</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="E7" t="s" s="6">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -288,7 +261,6 @@
     <hyperlink ref="E4" r:id="rId3"/>
     <hyperlink ref="E5" r:id="rId4"/>
     <hyperlink ref="E6" r:id="rId5"/>
-    <hyperlink ref="E7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>